<commit_message>
Feat: Dodanie skryptu generate_charts.py z interaktywnym wyborem okna oraz wygenerowanie wykresu
</commit_message>
<xml_diff>
--- a/data/Dane do analizy.xlsx
+++ b/data/Dane do analizy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dominikpopielarz/Desktop/zeglarstwo-analiza/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{378A40E7-984D-7644-9CDA-66DDFC9E0C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDDB2230-E52D-684E-8529-4E48BB0FDE98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="580" yWindow="660" windowWidth="28240" windowHeight="16660" activeTab="2" xr2:uid="{3439E772-BCE1-4E4B-8AE5-B5F16651E21C}"/>
+    <workbookView xWindow="580" yWindow="660" windowWidth="28240" windowHeight="16660" xr2:uid="{3439E772-BCE1-4E4B-8AE5-B5F16651E21C}"/>
   </bookViews>
   <sheets>
     <sheet name="Paweł" sheetId="1" r:id="rId1"/>
@@ -663,6 +663,9 @@
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1B8EBBBE-F867-9C46-9DF4-A432A2A7C2A1}" name="Tabela3" displayName="Tabela3" ref="A1:E35" totalsRowShown="0">
   <autoFilter ref="A1:E35" xr:uid="{1B8EBBBE-F867-9C46-9DF4-A432A2A7C2A1}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E35">
+    <sortCondition ref="A1:A35"/>
+  </sortState>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{8079B05C-AB9B-4C4D-8237-18BB3176B24A}" name="Sezon" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{BF1B558A-80E6-A54E-8677-8E6981E8FDC8}" name="Mc" dataDxfId="15"/>
@@ -2516,616 +2519,616 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="5">
-        <v>46143</v>
+        <v>44723</v>
       </c>
       <c r="B2" s="12">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="C2" s="12">
-        <v>182</v>
+        <v>41</v>
       </c>
       <c r="D2" s="12">
         <f>1-B2/C2</f>
-        <v>0.68131868131868134</v>
+        <v>0.36585365853658536</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="5">
-        <v>46186</v>
+        <v>44807</v>
       </c>
       <c r="B3" s="12">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="C3" s="12">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="D3" s="12">
-        <f t="shared" ref="D3:D35" si="0">1-B3/C3</f>
-        <v>0.90909090909090906</v>
+        <f>1-B3/C3</f>
+        <v>2.2222222222222254E-2</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
-        <v>46179</v>
+        <v>44835</v>
       </c>
       <c r="B4" s="12">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="C4" s="12">
         <v>48</v>
       </c>
       <c r="D4" s="12">
-        <f t="shared" si="0"/>
-        <v>0.79166666666666663</v>
+        <f>1-B4/C4</f>
+        <v>0.10416666666666663</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A5" s="5">
-        <v>46171</v>
+        <v>45073</v>
       </c>
       <c r="B5" s="12">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="C5" s="12">
-        <v>307</v>
+        <v>31</v>
       </c>
       <c r="D5" s="12">
-        <f t="shared" si="0"/>
-        <v>0.83387622149837137</v>
+        <f>1-B5/C5</f>
+        <v>0.70967741935483875</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
-        <v>46209</v>
+        <v>45092</v>
       </c>
       <c r="B6" s="12">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="C6" s="12">
-        <v>185</v>
+        <v>35</v>
       </c>
       <c r="D6" s="12">
-        <f t="shared" si="0"/>
-        <v>0.61621621621621614</v>
+        <f>1-B6/C6</f>
+        <v>0.17142857142857137</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>7</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="5">
-        <v>46223</v>
+        <v>45115</v>
       </c>
       <c r="B7" s="12">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C7" s="12">
-        <v>245</v>
+        <v>35</v>
       </c>
       <c r="D7" s="12">
-        <f t="shared" si="0"/>
-        <v>0.88163265306122451</v>
+        <f>1-B7/C7</f>
+        <v>0.74285714285714288</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="5">
-        <v>46260</v>
+        <v>45135</v>
       </c>
       <c r="B8" s="12">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C8" s="12">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="D8" s="12">
-        <f t="shared" si="0"/>
-        <v>0.77215189873417722</v>
+        <f>1-B8/C8</f>
+        <v>0.75862068965517238</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="68" x14ac:dyDescent="0.2">
       <c r="A9" s="5">
-        <v>46270</v>
+        <v>45148</v>
       </c>
       <c r="B9" s="12">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="C9" s="12">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="D9" s="12">
-        <f t="shared" si="0"/>
-        <v>0.85365853658536583</v>
+        <f>1-B9/C9</f>
+        <v>0.33333333333333337</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A10" s="5">
-        <v>46220</v>
+        <v>45149</v>
       </c>
       <c r="B10" s="12">
-        <v>105</v>
+        <v>21</v>
       </c>
       <c r="C10" s="12">
-        <v>362</v>
+        <v>55</v>
       </c>
       <c r="D10" s="12">
-        <f t="shared" si="0"/>
-        <v>0.70994475138121549</v>
+        <f>1-B10/C10</f>
+        <v>0.61818181818181817</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="5">
-        <v>45870</v>
+        <v>45169</v>
       </c>
       <c r="B11" s="12">
-        <v>148</v>
+        <v>11</v>
       </c>
       <c r="C11" s="12">
-        <v>289</v>
+        <v>44</v>
       </c>
       <c r="D11" s="12">
-        <f t="shared" si="0"/>
-        <v>0.48788927335640142</v>
+        <f>1-B11/C11</f>
+        <v>0.75</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="68" x14ac:dyDescent="0.2">
       <c r="A12" s="5">
-        <v>45815</v>
+        <v>45178</v>
       </c>
       <c r="B12" s="12">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C12" s="12">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="D12" s="12">
-        <f t="shared" si="0"/>
-        <v>0.77777777777777779</v>
+        <f>1-B12/C12</f>
+        <v>0.70967741935483875</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="5">
-        <v>45822</v>
+        <v>45199</v>
       </c>
       <c r="B13" s="12">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C13" s="12">
+        <v>37</v>
+      </c>
+      <c r="D13" s="12">
+        <f>1-B13/C13</f>
+        <v>0.6216216216216216</v>
+      </c>
+      <c r="E13" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="12">
-        <f t="shared" si="0"/>
-        <v>0.84615384615384615</v>
-      </c>
-      <c r="E13" s="11" t="s">
+    </row>
+    <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A14" s="5">
+        <v>45450</v>
+      </c>
+      <c r="B14" s="12">
+        <v>15</v>
+      </c>
+      <c r="C14" s="12">
+        <v>65</v>
+      </c>
+      <c r="D14" s="12">
+        <f>1-B14/C14</f>
+        <v>0.76923076923076916</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A15" s="5">
+        <v>45458</v>
+      </c>
+      <c r="B15" s="12">
+        <v>2</v>
+      </c>
+      <c r="C15" s="12">
+        <v>21</v>
+      </c>
+      <c r="D15" s="12">
+        <f>1-B15/C15</f>
+        <v>0.90476190476190477</v>
+      </c>
+      <c r="E15" s="11" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="68" x14ac:dyDescent="0.2">
-      <c r="A14" s="5">
-        <v>45877</v>
-      </c>
-      <c r="B14" s="12">
-        <v>10</v>
-      </c>
-      <c r="C14" s="12">
-        <v>58</v>
-      </c>
-      <c r="D14" s="12">
-        <f t="shared" si="0"/>
-        <v>0.82758620689655171</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A15" s="5">
-        <v>45896</v>
-      </c>
-      <c r="B15" s="12">
-        <v>50</v>
-      </c>
-      <c r="C15" s="12">
-        <v>79</v>
-      </c>
-      <c r="D15" s="12">
-        <f t="shared" si="0"/>
-        <v>0.36708860759493667</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="5">
-        <v>45450</v>
+        <v>45465</v>
       </c>
       <c r="B16" s="12">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C16" s="12">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="D16" s="12">
-        <f t="shared" si="0"/>
-        <v>0.76923076923076916</v>
+        <f>1-B16/C16</f>
+        <v>0.81818181818181812</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="5">
-        <v>45535</v>
+        <v>45479</v>
       </c>
       <c r="B17" s="12">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C17" s="12">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D17" s="12">
-        <f t="shared" si="0"/>
-        <v>0.67391304347826086</v>
+        <f>1-B17/C17</f>
+        <v>0.80555555555555558</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="5">
-        <v>45479</v>
+        <v>45493</v>
       </c>
       <c r="B18" s="12">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="C18" s="12">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="D18" s="12">
-        <f t="shared" si="0"/>
-        <v>0.80555555555555558</v>
+        <f>1-B18/C18</f>
+        <v>9.5238095238095233E-2</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A19" s="5">
-        <v>45465</v>
+        <v>45513</v>
       </c>
       <c r="B19" s="12">
+        <v>10</v>
+      </c>
+      <c r="C19" s="12">
+        <v>68</v>
+      </c>
+      <c r="D19" s="12">
+        <f>1-B19/C19</f>
+        <v>0.8529411764705882</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A20" s="5">
+        <v>45535</v>
+      </c>
+      <c r="B20" s="12">
+        <v>15</v>
+      </c>
+      <c r="C20" s="12">
+        <v>46</v>
+      </c>
+      <c r="D20" s="12">
+        <f>1-B20/C20</f>
+        <v>0.67391304347826086</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+      <c r="A21" s="5">
+        <v>45542</v>
+      </c>
+      <c r="B21" s="12">
+        <v>18</v>
+      </c>
+      <c r="C21" s="12">
+        <v>39</v>
+      </c>
+      <c r="D21" s="12">
+        <f>1-B21/C21</f>
+        <v>0.53846153846153844</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A22" s="5">
+        <v>45815</v>
+      </c>
+      <c r="B22" s="12">
+        <v>14</v>
+      </c>
+      <c r="C22" s="12">
+        <v>63</v>
+      </c>
+      <c r="D22" s="12">
+        <f>1-B22/C22</f>
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A23" s="5">
+        <v>45822</v>
+      </c>
+      <c r="B23" s="12">
         <v>6</v>
       </c>
-      <c r="C19" s="12">
-        <v>33</v>
-      </c>
-      <c r="D19" s="12">
-        <f t="shared" si="0"/>
-        <v>0.81818181818181812</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="68" x14ac:dyDescent="0.2">
-      <c r="A20" s="5">
-        <v>45542</v>
-      </c>
-      <c r="B20" s="12">
-        <v>18</v>
-      </c>
-      <c r="C20" s="12">
+      <c r="C23" s="12">
         <v>39</v>
       </c>
-      <c r="D20" s="12">
-        <f t="shared" si="0"/>
-        <v>0.53846153846153844</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A21" s="5">
-        <v>45458</v>
-      </c>
-      <c r="B21" s="12">
-        <v>2</v>
-      </c>
-      <c r="C21" s="12">
-        <v>21</v>
-      </c>
-      <c r="D21" s="12">
-        <f t="shared" si="0"/>
-        <v>0.90476190476190477</v>
-      </c>
-      <c r="E21" s="11" t="s">
+      <c r="D23" s="12">
+        <f>1-B23/C23</f>
+        <v>0.84615384615384615</v>
+      </c>
+      <c r="E23" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" s="5">
-        <v>45493</v>
-      </c>
-      <c r="B22" s="12">
+    <row r="24" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A24" s="5">
+        <v>45855</v>
+      </c>
+      <c r="B24" s="12">
+        <v>105</v>
+      </c>
+      <c r="C24" s="12">
+        <v>362</v>
+      </c>
+      <c r="D24" s="12">
+        <f>1-B24/C24</f>
+        <v>0.70994475138121549</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A25" s="5">
+        <v>45870</v>
+      </c>
+      <c r="B25" s="12">
+        <v>148</v>
+      </c>
+      <c r="C25" s="12">
+        <v>289</v>
+      </c>
+      <c r="D25" s="12">
+        <f>1-B25/C25</f>
+        <v>0.48788927335640142</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+      <c r="A26" s="5">
+        <v>45877</v>
+      </c>
+      <c r="B26" s="12">
+        <v>10</v>
+      </c>
+      <c r="C26" s="12">
+        <v>58</v>
+      </c>
+      <c r="D26" s="12">
+        <f>1-B26/C26</f>
+        <v>0.82758620689655171</v>
+      </c>
+      <c r="E26" s="11" t="s">
         <v>19</v>
-      </c>
-      <c r="C22" s="12">
-        <v>21</v>
-      </c>
-      <c r="D22" s="12">
-        <f t="shared" si="0"/>
-        <v>9.5238095238095233E-2</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A23" s="5">
-        <v>45513</v>
-      </c>
-      <c r="B23" s="12">
-        <v>10</v>
-      </c>
-      <c r="C23" s="12">
-        <v>68</v>
-      </c>
-      <c r="D23" s="12">
-        <f t="shared" si="0"/>
-        <v>0.8529411764705882</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="5">
-        <v>45169</v>
-      </c>
-      <c r="B24" s="12">
-        <v>11</v>
-      </c>
-      <c r="C24" s="12">
-        <v>44</v>
-      </c>
-      <c r="D24" s="12">
-        <f t="shared" si="0"/>
-        <v>0.75</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="68" x14ac:dyDescent="0.2">
-      <c r="A25" s="5">
-        <v>45148</v>
-      </c>
-      <c r="B25" s="12">
-        <v>52</v>
-      </c>
-      <c r="C25" s="12">
-        <v>78</v>
-      </c>
-      <c r="D25" s="12">
-        <f t="shared" si="0"/>
-        <v>0.33333333333333337</v>
-      </c>
-      <c r="E25" s="11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A26" s="5">
-        <v>45115</v>
-      </c>
-      <c r="B26" s="12">
-        <v>9</v>
-      </c>
-      <c r="C26" s="12">
-        <v>35</v>
-      </c>
-      <c r="D26" s="12">
-        <f t="shared" si="0"/>
-        <v>0.74285714285714288</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A27" s="5">
-        <v>45073</v>
+        <v>45896</v>
       </c>
       <c r="B27" s="12">
-        <v>9</v>
+        <v>50</v>
       </c>
       <c r="C27" s="12">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="D27" s="12">
-        <f t="shared" si="0"/>
-        <v>0.70967741935483875</v>
+        <f>1-B27/C27</f>
+        <v>0.36708860759493667</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="5">
-        <v>45178</v>
+        <v>46143</v>
       </c>
       <c r="B28" s="12">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="C28" s="12">
-        <v>31</v>
+        <v>182</v>
       </c>
       <c r="D28" s="12">
-        <f t="shared" si="0"/>
-        <v>0.70967741935483875</v>
+        <f>1-B28/C28</f>
+        <v>0.68131868131868134</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>37</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A29" s="5">
-        <v>45092</v>
+        <v>46171</v>
       </c>
       <c r="B29" s="12">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="C29" s="12">
-        <v>35</v>
+        <v>307</v>
       </c>
       <c r="D29" s="12">
-        <f t="shared" si="0"/>
-        <v>0.17142857142857137</v>
+        <f>1-B29/C29</f>
+        <v>0.83387622149837137</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="5">
-        <v>45149</v>
+        <v>46179</v>
       </c>
       <c r="B30" s="12">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C30" s="12">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D30" s="12">
-        <f t="shared" si="0"/>
-        <v>0.61818181818181817</v>
+        <f>1-B30/C30</f>
+        <v>0.79166666666666663</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>38</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" s="5">
-        <v>45135</v>
+        <v>46186</v>
       </c>
       <c r="B31" s="12">
+        <v>3</v>
+      </c>
+      <c r="C31" s="12">
+        <v>33</v>
+      </c>
+      <c r="D31" s="12">
+        <f>1-B31/C31</f>
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="E31" s="11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A32" s="5">
+        <v>46209</v>
+      </c>
+      <c r="B32" s="12">
+        <v>71</v>
+      </c>
+      <c r="C32" s="12">
+        <v>185</v>
+      </c>
+      <c r="D32" s="12">
+        <f>1-B32/C32</f>
+        <v>0.61621621621621614</v>
+      </c>
+      <c r="E32" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C31" s="12">
+    </row>
+    <row r="33" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A33" s="5">
+        <v>46223</v>
+      </c>
+      <c r="B33" s="12">
         <v>29</v>
       </c>
-      <c r="D31" s="12">
-        <f t="shared" si="0"/>
-        <v>0.75862068965517238</v>
-      </c>
-      <c r="E31" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A32" s="5">
-        <v>45199</v>
-      </c>
-      <c r="B32" s="12">
-        <v>14</v>
-      </c>
-      <c r="C32" s="12">
-        <v>37</v>
-      </c>
-      <c r="D32" s="12">
-        <f t="shared" si="0"/>
-        <v>0.6216216216216216</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A33" s="5">
-        <v>44807</v>
-      </c>
-      <c r="B33" s="12">
-        <v>44</v>
-      </c>
       <c r="C33" s="12">
-        <v>45</v>
+        <v>245</v>
       </c>
       <c r="D33" s="12">
-        <f t="shared" si="0"/>
-        <v>2.2222222222222254E-2</v>
+        <f>1-B33/C33</f>
+        <v>0.88163265306122451</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="5">
-        <v>44723</v>
+        <v>46260</v>
       </c>
       <c r="B34" s="12">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C34" s="12">
+        <v>79</v>
+      </c>
+      <c r="D34" s="12">
+        <f>1-B34/C34</f>
+        <v>0.77215189873417722</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A35" s="5">
+        <v>46270</v>
+      </c>
+      <c r="B35" s="12">
+        <v>6</v>
+      </c>
+      <c r="C35" s="12">
         <v>41</v>
       </c>
-      <c r="D34" s="12">
-        <f t="shared" si="0"/>
-        <v>0.36585365853658536</v>
-      </c>
-      <c r="E34" s="11" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A35" s="5">
-        <v>44835</v>
-      </c>
-      <c r="B35" s="12">
-        <v>43</v>
-      </c>
-      <c r="C35" s="12">
-        <v>48</v>
-      </c>
       <c r="D35" s="12">
-        <f t="shared" si="0"/>
-        <v>0.10416666666666663</v>
+        <f>1-B35/C35</f>
+        <v>0.85365853658536583</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -3143,40 +3146,40 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" display="https://portal2.psko.pl/regaty/puchar-ks-zatoka-puck---opp-b-2026" xr:uid="{92C73110-FF61-FD4C-8FB2-E1E9880D5E49}"/>
-    <hyperlink ref="E3" r:id="rId2" display="https://portal2.psko.pl/regaty/puchar-safege-2026" xr:uid="{E7479D72-96F3-4142-B9E2-CFAAEF2F4308}"/>
-    <hyperlink ref="E4" r:id="rId3" display="https://portal2.psko.pl/regaty/puchar-tkz-torun-2026" xr:uid="{A4A90A71-B48D-4044-98D3-58E1C0C297B7}"/>
-    <hyperlink ref="E5" r:id="rId4" display="https://portal2.psko.pl/regaty/42-regaty-pomaranczowe-eliminacja-mpm-2026" xr:uid="{467B49A7-53C9-FC4E-8183-750BF6B3C2BA}"/>
-    <hyperlink ref="E6" r:id="rId5" display="https://portal2.psko.pl/regaty/puchar-trenerow-klasy-optimist-gr-b-w-ramach-lotto-gdynia-sailing-days-2026" xr:uid="{07ECACB3-2A2C-3B44-A440-4625C6591C0A}"/>
-    <hyperlink ref="E7" r:id="rId6" display="https://portal2.psko.pl/regaty/puchar-jeziora-zegrzynskiego-eliminacja-mistrzostw-polski-mlodzikow-2026" xr:uid="{ABA083B1-F47B-0A4B-BC2D-2336D02A1041}"/>
-    <hyperlink ref="E8" r:id="rId7" display="https://portal2.psko.pl/regaty/mistrzostwa-polski-mlodzikow-2026" xr:uid="{964199F3-0EF1-3647-8203-25F709D96D44}"/>
-    <hyperlink ref="E9" r:id="rId8" display="https://portal2.psko.pl/regaty/puchar-znina-2026" xr:uid="{2060568C-C545-5444-A51B-36272B320B9D}"/>
-    <hyperlink ref="E10" r:id="rId9" display="https://portal2.psko.pl/regaty/kinder-joy-of-moving,--puchar-trenerow,-eliminacja-mistrzostw-polski-mlodzikow-2025" xr:uid="{AB453DBC-7619-8941-B9C6-CD7096DF6622}"/>
-    <hyperlink ref="E11" r:id="rId10" display="https://portal2.psko.pl/regaty/srebrny-zagiel-optimista,-eliminacja-mistrzostw-polski-mlodzikow-2025" xr:uid="{37954E7F-16DC-2644-A0A1-2242ED79FC08}"/>
-    <hyperlink ref="E12" r:id="rId11" display="https://portal2.psko.pl/regaty/puchar-tkz-torun-2025" xr:uid="{132F47D0-28B6-9844-B408-98668C211D71}"/>
-    <hyperlink ref="E13" r:id="rId12" display="https://portal2.psko.pl/regaty/puchar-safege-2025" xr:uid="{A3125F74-D9E3-4049-838B-EA2AECF7E0DA}"/>
-    <hyperlink ref="E14" r:id="rId13" display="https://portal2.psko.pl/regaty/zagle-2025,-mistrzostwa-polskiego-stowarzyszenia-klasy-optimist-u-12-2025" xr:uid="{D24DBCED-0DB1-1647-A97D-A610123BB336}"/>
-    <hyperlink ref="E16" r:id="rId14" display="https://portal2.psko.pl/regaty/puchar-tkz-2024" xr:uid="{E29A3531-D26C-2245-AC6E-E0AD3B50F0F7}"/>
-    <hyperlink ref="E17" r:id="rId15" display="https://portal2.psko.pl/regaty/puchar-znina-2024" xr:uid="{47B4D731-C872-8745-95F4-CF57161348EC}"/>
-    <hyperlink ref="E18" r:id="rId16" display="https://portal2.psko.pl/regaty/ix-regaty-o-puchar-columba-2024" xr:uid="{53F728DC-64C1-8C47-9AF1-A9F2860C8FB7}"/>
-    <hyperlink ref="E19" r:id="rId17" display="https://portal2.psko.pl/regaty/regaty-o-puchar-kormorana-2024" xr:uid="{3B592B7A-2CC5-A849-AA59-8FD22C5EB27D}"/>
-    <hyperlink ref="E20" r:id="rId18" display="https://portal2.psko.pl/regaty/xiii-regaty-optysiowe-2024" xr:uid="{F11FAF75-BB49-AD40-9144-CA4720533331}"/>
-    <hyperlink ref="E21" r:id="rId19" display="https://portal2.psko.pl/regaty/puchar-safege-2024" xr:uid="{CCCAE64D-B7D5-9E44-9FDF-24044A290F73}"/>
-    <hyperlink ref="E22" r:id="rId20" display="https://portal2.psko.pl/regaty/10-baltycki-puchar-klas-2024" xr:uid="{028FB2BD-418C-F843-9055-95C9F4ADC43A}"/>
-    <hyperlink ref="E23" r:id="rId21" display="https://portal2.psko.pl/regaty/zagle-2024-xix-mistrzostwa-polskiego-stowarzyszenia-klasy-optimist-do-lat-11-2024" xr:uid="{0359F2E5-B85C-9F45-95BF-4EA88005DDE9}"/>
-    <hyperlink ref="E24" r:id="rId22" display="https://portal2.psko.pl/regaty/puchar-znina-2023" xr:uid="{9F039AC2-AD4F-5B4D-9FA0-3B3A805D8377}"/>
-    <hyperlink ref="E25" r:id="rId23" display="https://portal2.psko.pl/regaty/zagle-2023-xxi-ogolnopolskie-regaty-o-puchar-ziemi-zlocienieckiej-2023" xr:uid="{BBB97408-8771-7447-AC55-388C51BD5DC2}"/>
-    <hyperlink ref="E26" r:id="rId24" display="https://portal2.psko.pl/regaty/viii-regaty-o-puchar-columba-2023" xr:uid="{C567056E-3FE1-8941-8D4C-5A83C8E3CF9B}"/>
-    <hyperlink ref="E27" r:id="rId25" display="https://portal2.psko.pl/regaty/-puchar-burmistrza-czluchowa-2023" xr:uid="{7C21A92D-AE21-4E40-B071-E8EDFD54E41A}"/>
-    <hyperlink ref="E28" r:id="rId26" display="https://portal2.psko.pl/regaty/xii-regaty-optysiowe-2023" xr:uid="{B1CAFCD6-8F8B-B149-BA9D-630DA0A15376}"/>
-    <hyperlink ref="E29" r:id="rId27" display="https://portal2.psko.pl/regaty/puchar-safege-2023" xr:uid="{252DBE58-9C70-664B-895A-421A80C95188}"/>
-    <hyperlink ref="E30" r:id="rId28" display="https://portal2.psko.pl/regaty/zagle-2023-xvii-mistrzostwa-polskiego-stowarzyszenia-klasy-optimist-do-lat-11-2023" xr:uid="{B9EDE181-5187-F049-A8D2-85FA88B88B7E}"/>
-    <hyperlink ref="E31" r:id="rId29" display="https://portal2.psko.pl/regaty/mistrzostwa-psko-do-lat-9-2023" xr:uid="{DA055ECB-04F7-5044-9D8D-FD45572724F9}"/>
-    <hyperlink ref="E32" r:id="rId30" display="https://portal2.psko.pl/regaty/mmm---pom,-kuj-pom-2023" xr:uid="{4C061EDF-E374-FF4B-8660-9D4F067CE200}"/>
-    <hyperlink ref="E33" r:id="rId31" display="https://portal2.psko.pl/regaty/puchar-znina-2022" xr:uid="{43C8F71B-1352-3249-9929-4327C8627DEE}"/>
-    <hyperlink ref="E34" r:id="rId32" display="https://portal2.psko.pl/regaty/puchar-safege-2022" xr:uid="{9F4BEEB4-C811-F547-B85F-EBD2965EEED4}"/>
-    <hyperlink ref="E35" r:id="rId33" display="https://portal2.psko.pl/regaty/mmm---pom-i-kuj-pom-2022" xr:uid="{B3F9DF80-8CD1-CB41-AE26-4896F70DE7A5}"/>
-    <hyperlink ref="E15" r:id="rId34" display="https://portal2.psko.pl/regaty/puchar-mazur,-mistrzostwa-polski-mlodzikow-2025" xr:uid="{E8F825DB-C9F5-C04C-899C-B22DD64B7FD8}"/>
+    <hyperlink ref="E28" r:id="rId1" display="https://portal2.psko.pl/regaty/puchar-ks-zatoka-puck---opp-b-2026" xr:uid="{92C73110-FF61-FD4C-8FB2-E1E9880D5E49}"/>
+    <hyperlink ref="E31" r:id="rId2" display="https://portal2.psko.pl/regaty/puchar-safege-2026" xr:uid="{E7479D72-96F3-4142-B9E2-CFAAEF2F4308}"/>
+    <hyperlink ref="E30" r:id="rId3" display="https://portal2.psko.pl/regaty/puchar-tkz-torun-2026" xr:uid="{A4A90A71-B48D-4044-98D3-58E1C0C297B7}"/>
+    <hyperlink ref="E29" r:id="rId4" display="https://portal2.psko.pl/regaty/42-regaty-pomaranczowe-eliminacja-mpm-2026" xr:uid="{467B49A7-53C9-FC4E-8183-750BF6B3C2BA}"/>
+    <hyperlink ref="E32" r:id="rId5" display="https://portal2.psko.pl/regaty/puchar-trenerow-klasy-optimist-gr-b-w-ramach-lotto-gdynia-sailing-days-2026" xr:uid="{07ECACB3-2A2C-3B44-A440-4625C6591C0A}"/>
+    <hyperlink ref="E33" r:id="rId6" display="https://portal2.psko.pl/regaty/puchar-jeziora-zegrzynskiego-eliminacja-mistrzostw-polski-mlodzikow-2026" xr:uid="{ABA083B1-F47B-0A4B-BC2D-2336D02A1041}"/>
+    <hyperlink ref="E34" r:id="rId7" display="https://portal2.psko.pl/regaty/mistrzostwa-polski-mlodzikow-2026" xr:uid="{964199F3-0EF1-3647-8203-25F709D96D44}"/>
+    <hyperlink ref="E35" r:id="rId8" display="https://portal2.psko.pl/regaty/puchar-znina-2026" xr:uid="{2060568C-C545-5444-A51B-36272B320B9D}"/>
+    <hyperlink ref="E24" r:id="rId9" display="https://portal2.psko.pl/regaty/kinder-joy-of-moving,--puchar-trenerow,-eliminacja-mistrzostw-polski-mlodzikow-2025" xr:uid="{AB453DBC-7619-8941-B9C6-CD7096DF6622}"/>
+    <hyperlink ref="E25" r:id="rId10" display="https://portal2.psko.pl/regaty/srebrny-zagiel-optimista,-eliminacja-mistrzostw-polski-mlodzikow-2025" xr:uid="{37954E7F-16DC-2644-A0A1-2242ED79FC08}"/>
+    <hyperlink ref="E22" r:id="rId11" display="https://portal2.psko.pl/regaty/puchar-tkz-torun-2025" xr:uid="{132F47D0-28B6-9844-B408-98668C211D71}"/>
+    <hyperlink ref="E23" r:id="rId12" display="https://portal2.psko.pl/regaty/puchar-safege-2025" xr:uid="{A3125F74-D9E3-4049-838B-EA2AECF7E0DA}"/>
+    <hyperlink ref="E26" r:id="rId13" display="https://portal2.psko.pl/regaty/zagle-2025,-mistrzostwa-polskiego-stowarzyszenia-klasy-optimist-u-12-2025" xr:uid="{D24DBCED-0DB1-1647-A97D-A610123BB336}"/>
+    <hyperlink ref="E14" r:id="rId14" display="https://portal2.psko.pl/regaty/puchar-tkz-2024" xr:uid="{E29A3531-D26C-2245-AC6E-E0AD3B50F0F7}"/>
+    <hyperlink ref="E20" r:id="rId15" display="https://portal2.psko.pl/regaty/puchar-znina-2024" xr:uid="{47B4D731-C872-8745-95F4-CF57161348EC}"/>
+    <hyperlink ref="E17" r:id="rId16" display="https://portal2.psko.pl/regaty/ix-regaty-o-puchar-columba-2024" xr:uid="{53F728DC-64C1-8C47-9AF1-A9F2860C8FB7}"/>
+    <hyperlink ref="E16" r:id="rId17" display="https://portal2.psko.pl/regaty/regaty-o-puchar-kormorana-2024" xr:uid="{3B592B7A-2CC5-A849-AA59-8FD22C5EB27D}"/>
+    <hyperlink ref="E21" r:id="rId18" display="https://portal2.psko.pl/regaty/xiii-regaty-optysiowe-2024" xr:uid="{F11FAF75-BB49-AD40-9144-CA4720533331}"/>
+    <hyperlink ref="E15" r:id="rId19" display="https://portal2.psko.pl/regaty/puchar-safege-2024" xr:uid="{CCCAE64D-B7D5-9E44-9FDF-24044A290F73}"/>
+    <hyperlink ref="E18" r:id="rId20" display="https://portal2.psko.pl/regaty/10-baltycki-puchar-klas-2024" xr:uid="{028FB2BD-418C-F843-9055-95C9F4ADC43A}"/>
+    <hyperlink ref="E19" r:id="rId21" display="https://portal2.psko.pl/regaty/zagle-2024-xix-mistrzostwa-polskiego-stowarzyszenia-klasy-optimist-do-lat-11-2024" xr:uid="{0359F2E5-B85C-9F45-95BF-4EA88005DDE9}"/>
+    <hyperlink ref="E11" r:id="rId22" display="https://portal2.psko.pl/regaty/puchar-znina-2023" xr:uid="{9F039AC2-AD4F-5B4D-9FA0-3B3A805D8377}"/>
+    <hyperlink ref="E9" r:id="rId23" display="https://portal2.psko.pl/regaty/zagle-2023-xxi-ogolnopolskie-regaty-o-puchar-ziemi-zlocienieckiej-2023" xr:uid="{BBB97408-8771-7447-AC55-388C51BD5DC2}"/>
+    <hyperlink ref="E7" r:id="rId24" display="https://portal2.psko.pl/regaty/viii-regaty-o-puchar-columba-2023" xr:uid="{C567056E-3FE1-8941-8D4C-5A83C8E3CF9B}"/>
+    <hyperlink ref="E5" r:id="rId25" display="https://portal2.psko.pl/regaty/-puchar-burmistrza-czluchowa-2023" xr:uid="{7C21A92D-AE21-4E40-B071-E8EDFD54E41A}"/>
+    <hyperlink ref="E12" r:id="rId26" display="https://portal2.psko.pl/regaty/xii-regaty-optysiowe-2023" xr:uid="{B1CAFCD6-8F8B-B149-BA9D-630DA0A15376}"/>
+    <hyperlink ref="E6" r:id="rId27" display="https://portal2.psko.pl/regaty/puchar-safege-2023" xr:uid="{252DBE58-9C70-664B-895A-421A80C95188}"/>
+    <hyperlink ref="E10" r:id="rId28" display="https://portal2.psko.pl/regaty/zagle-2023-xvii-mistrzostwa-polskiego-stowarzyszenia-klasy-optimist-do-lat-11-2023" xr:uid="{B9EDE181-5187-F049-A8D2-85FA88B88B7E}"/>
+    <hyperlink ref="E8" r:id="rId29" display="https://portal2.psko.pl/regaty/mistrzostwa-psko-do-lat-9-2023" xr:uid="{DA055ECB-04F7-5044-9D8D-FD45572724F9}"/>
+    <hyperlink ref="E13" r:id="rId30" display="https://portal2.psko.pl/regaty/mmm---pom,-kuj-pom-2023" xr:uid="{4C061EDF-E374-FF4B-8660-9D4F067CE200}"/>
+    <hyperlink ref="E3" r:id="rId31" display="https://portal2.psko.pl/regaty/puchar-znina-2022" xr:uid="{43C8F71B-1352-3249-9929-4327C8627DEE}"/>
+    <hyperlink ref="E2" r:id="rId32" display="https://portal2.psko.pl/regaty/puchar-safege-2022" xr:uid="{9F4BEEB4-C811-F547-B85F-EBD2965EEED4}"/>
+    <hyperlink ref="E4" r:id="rId33" display="https://portal2.psko.pl/regaty/mmm---pom-i-kuj-pom-2022" xr:uid="{B3F9DF80-8CD1-CB41-AE26-4896F70DE7A5}"/>
+    <hyperlink ref="E27" r:id="rId34" display="https://portal2.psko.pl/regaty/puchar-mazur,-mistrzostwa-polski-mlodzikow-2025" xr:uid="{E8F825DB-C9F5-C04C-899C-B22DD64B7FD8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(analytics): dodano wskaźnik CV oraz moduł analizy pojedynczych regat
</commit_message>
<xml_diff>
--- a/data/Dane do analizy.xlsx
+++ b/data/Dane do analizy.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dominikpopielarz/Desktop/zeglarstwo-analiza/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDDB2230-E52D-684E-8529-4E48BB0FDE98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB66B94E-FC35-8B48-A7AE-23F2B3F9DEBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="580" yWindow="660" windowWidth="28240" windowHeight="16660" xr2:uid="{3439E772-BCE1-4E4B-8AE5-B5F16651E21C}"/>
+    <workbookView xWindow="580" yWindow="660" windowWidth="28240" windowHeight="16660" activeTab="2" xr2:uid="{3439E772-BCE1-4E4B-8AE5-B5F16651E21C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Paweł" sheetId="1" r:id="rId1"/>
-    <sheet name="Wojciech" sheetId="2" r:id="rId2"/>
-    <sheet name="Lidia" sheetId="3" r:id="rId3"/>
+    <sheet name="Paweł Fanslau" sheetId="1" r:id="rId1"/>
+    <sheet name="Wojciech Krasoń" sheetId="2" r:id="rId2"/>
+    <sheet name="Lidia Zdzierak" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -417,6 +417,86 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color rgb="FF3F4254"/>
+        <name val="Helvetica"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color rgb="FF3F4254"/>
+        <name val="Helvetica"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color rgb="FF3F4254"/>
+        <name val="Helvetica"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color rgb="FF3F4254"/>
+        <name val="Helvetica"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="d/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -531,86 +611,6 @@
         <scheme val="none"/>
       </font>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color rgb="FF3F4254"/>
-        <name val="Helvetica"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color rgb="FF3F4254"/>
-        <name val="Helvetica"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color rgb="FF3F4254"/>
-        <name val="Helvetica"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color rgb="FF3F4254"/>
-        <name val="Helvetica"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="d/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -625,36 +625,36 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CFB21AE2-C426-9747-9257-0814E9080719}" name="Tabela1" displayName="Tabela1" ref="A1:E29" totalsRowShown="0" headerRowDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CFB21AE2-C426-9747-9257-0814E9080719}" name="Tabela1" displayName="Tabela1" ref="A1:E29" totalsRowShown="0" headerRowDxfId="16">
   <autoFilter ref="A1:E29" xr:uid="{CFB21AE2-C426-9747-9257-0814E9080719}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E29">
     <sortCondition ref="A1:A29"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{956B7CC9-9152-A048-8B12-BCB6991D9AAA}" name="Data rozpoczęcia" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{AC41BCE8-5552-2B43-B1CF-B9305E3E7BE6}" name="Mc" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{39408C63-1019-3046-8C62-0A298F181A8A}" name="L. uczestników" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{43BBAFEF-D7D9-2F48-8318-7DBE2A7B7862}" name="Normalizacja" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{B9192BB7-8EBE-AA41-8653-42F92ED5BD64}" name="Nazwa regat" dataDxfId="6" dataCellStyle="Hiperłącze"/>
+    <tableColumn id="1" xr3:uid="{956B7CC9-9152-A048-8B12-BCB6991D9AAA}" name="Data rozpoczęcia" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{AC41BCE8-5552-2B43-B1CF-B9305E3E7BE6}" name="Mc" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{39408C63-1019-3046-8C62-0A298F181A8A}" name="L. uczestników" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{43BBAFEF-D7D9-2F48-8318-7DBE2A7B7862}" name="Normalizacja" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{B9192BB7-8EBE-AA41-8653-42F92ED5BD64}" name="Nazwa regat" dataDxfId="11" dataCellStyle="Hiperłącze"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1144380-6137-2144-A037-93D272C56562}" name="Tabela2" displayName="Tabela2" ref="A1:E47" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1144380-6137-2144-A037-93D272C56562}" name="Tabela2" displayName="Tabela2" ref="A1:E47" totalsRowShown="0" headerRowDxfId="10">
   <autoFilter ref="A1:E47" xr:uid="{B1144380-6137-2144-A037-93D272C56562}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E47">
     <sortCondition ref="A1:A47"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{07E02266-9FCA-1C41-8ABF-B8F7F6DE5A15}" name="Data rozpoczęcia" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{0A432EEA-7C25-D44D-80AC-96A29CE8939E}" name="Mc" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{09460BCC-0A03-0B4B-9B30-CD1819313075}" name="L. uczestników" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{09664402-41A6-4A46-958B-5B7C3E90FFB4}" name="normalizacja" dataDxfId="1">
+    <tableColumn id="1" xr3:uid="{07E02266-9FCA-1C41-8ABF-B8F7F6DE5A15}" name="Data rozpoczęcia" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{0A432EEA-7C25-D44D-80AC-96A29CE8939E}" name="Mc" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{09460BCC-0A03-0B4B-9B30-CD1819313075}" name="L. uczestników" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{09664402-41A6-4A46-958B-5B7C3E90FFB4}" name="normalizacja" dataDxfId="6">
       <calculatedColumnFormula>1-B2/C2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{4B968B31-EB32-8442-9C4B-7C831482B77B}" name="Nazwa regat" dataDxfId="0" dataCellStyle="Hiperłącze"/>
+    <tableColumn id="5" xr3:uid="{4B968B31-EB32-8442-9C4B-7C831482B77B}" name="Nazwa regat" dataDxfId="5" dataCellStyle="Hiperłącze"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -667,13 +667,13 @@
     <sortCondition ref="A1:A35"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{8079B05C-AB9B-4C4D-8237-18BB3176B24A}" name="Sezon" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{BF1B558A-80E6-A54E-8677-8E6981E8FDC8}" name="Mc" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{4AB3F412-CE48-6845-B58B-E59529C664C6}" name="L. uczestników" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{057D4DC5-E90A-EF45-8EFB-40A6D7149979}" name="normalizacja" dataDxfId="13">
+    <tableColumn id="1" xr3:uid="{8079B05C-AB9B-4C4D-8237-18BB3176B24A}" name="Sezon" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{BF1B558A-80E6-A54E-8677-8E6981E8FDC8}" name="Mc" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{4AB3F412-CE48-6845-B58B-E59529C664C6}" name="L. uczestników" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{057D4DC5-E90A-EF45-8EFB-40A6D7149979}" name="normalizacja" dataDxfId="1">
       <calculatedColumnFormula>1-B2/C2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{D302BD72-198A-D042-A525-74F7CE88B9A3}" name="Nazwa regat" dataDxfId="12" dataCellStyle="Hiperłącze"/>
+    <tableColumn id="5" xr3:uid="{D302BD72-198A-D042-A525-74F7CE88B9A3}" name="Nazwa regat" dataDxfId="0" dataCellStyle="Hiperłącze"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2530,7 +2530,7 @@
         <v>41</v>
       </c>
       <c r="D2" s="12">
-        <f>1-B2/C2</f>
+        <f t="shared" ref="D2:D35" si="0">1-B2/C2</f>
         <v>0.36585365853658536</v>
       </c>
       <c r="E2" s="11" t="s">
@@ -2548,7 +2548,7 @@
         <v>45</v>
       </c>
       <c r="D3" s="12">
-        <f>1-B3/C3</f>
+        <f t="shared" si="0"/>
         <v>2.2222222222222254E-2</v>
       </c>
       <c r="E3" s="11" t="s">
@@ -2566,7 +2566,7 @@
         <v>48</v>
       </c>
       <c r="D4" s="12">
-        <f>1-B4/C4</f>
+        <f t="shared" si="0"/>
         <v>0.10416666666666663</v>
       </c>
       <c r="E4" s="11" t="s">
@@ -2584,7 +2584,7 @@
         <v>31</v>
       </c>
       <c r="D5" s="12">
-        <f>1-B5/C5</f>
+        <f t="shared" si="0"/>
         <v>0.70967741935483875</v>
       </c>
       <c r="E5" s="11" t="s">
@@ -2602,7 +2602,7 @@
         <v>35</v>
       </c>
       <c r="D6" s="12">
-        <f>1-B6/C6</f>
+        <f t="shared" si="0"/>
         <v>0.17142857142857137</v>
       </c>
       <c r="E6" s="11" t="s">
@@ -2620,7 +2620,7 @@
         <v>35</v>
       </c>
       <c r="D7" s="12">
-        <f>1-B7/C7</f>
+        <f t="shared" si="0"/>
         <v>0.74285714285714288</v>
       </c>
       <c r="E7" s="11" t="s">
@@ -2638,7 +2638,7 @@
         <v>29</v>
       </c>
       <c r="D8" s="12">
-        <f>1-B8/C8</f>
+        <f t="shared" si="0"/>
         <v>0.75862068965517238</v>
       </c>
       <c r="E8" s="11" t="s">
@@ -2656,7 +2656,7 @@
         <v>78</v>
       </c>
       <c r="D9" s="12">
-        <f>1-B9/C9</f>
+        <f t="shared" si="0"/>
         <v>0.33333333333333337</v>
       </c>
       <c r="E9" s="11" t="s">
@@ -2674,7 +2674,7 @@
         <v>55</v>
       </c>
       <c r="D10" s="12">
-        <f>1-B10/C10</f>
+        <f t="shared" si="0"/>
         <v>0.61818181818181817</v>
       </c>
       <c r="E10" s="11" t="s">
@@ -2692,7 +2692,7 @@
         <v>44</v>
       </c>
       <c r="D11" s="12">
-        <f>1-B11/C11</f>
+        <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
       <c r="E11" s="11" t="s">
@@ -2710,7 +2710,7 @@
         <v>31</v>
       </c>
       <c r="D12" s="12">
-        <f>1-B12/C12</f>
+        <f t="shared" si="0"/>
         <v>0.70967741935483875</v>
       </c>
       <c r="E12" s="11" t="s">
@@ -2728,7 +2728,7 @@
         <v>37</v>
       </c>
       <c r="D13" s="12">
-        <f>1-B13/C13</f>
+        <f t="shared" si="0"/>
         <v>0.6216216216216216</v>
       </c>
       <c r="E13" s="11" t="s">
@@ -2746,7 +2746,7 @@
         <v>65</v>
       </c>
       <c r="D14" s="12">
-        <f>1-B14/C14</f>
+        <f t="shared" si="0"/>
         <v>0.76923076923076916</v>
       </c>
       <c r="E14" s="11" t="s">
@@ -2764,7 +2764,7 @@
         <v>21</v>
       </c>
       <c r="D15" s="12">
-        <f>1-B15/C15</f>
+        <f t="shared" si="0"/>
         <v>0.90476190476190477</v>
       </c>
       <c r="E15" s="11" t="s">
@@ -2782,7 +2782,7 @@
         <v>33</v>
       </c>
       <c r="D16" s="12">
-        <f>1-B16/C16</f>
+        <f t="shared" si="0"/>
         <v>0.81818181818181812</v>
       </c>
       <c r="E16" s="11" t="s">
@@ -2800,7 +2800,7 @@
         <v>36</v>
       </c>
       <c r="D17" s="12">
-        <f>1-B17/C17</f>
+        <f t="shared" si="0"/>
         <v>0.80555555555555558</v>
       </c>
       <c r="E17" s="11" t="s">
@@ -2818,7 +2818,7 @@
         <v>21</v>
       </c>
       <c r="D18" s="12">
-        <f>1-B18/C18</f>
+        <f t="shared" si="0"/>
         <v>9.5238095238095233E-2</v>
       </c>
       <c r="E18" s="11" t="s">
@@ -2836,7 +2836,7 @@
         <v>68</v>
       </c>
       <c r="D19" s="12">
-        <f>1-B19/C19</f>
+        <f t="shared" si="0"/>
         <v>0.8529411764705882</v>
       </c>
       <c r="E19" s="11" t="s">
@@ -2854,7 +2854,7 @@
         <v>46</v>
       </c>
       <c r="D20" s="12">
-        <f>1-B20/C20</f>
+        <f t="shared" si="0"/>
         <v>0.67391304347826086</v>
       </c>
       <c r="E20" s="11" t="s">
@@ -2872,7 +2872,7 @@
         <v>39</v>
       </c>
       <c r="D21" s="12">
-        <f>1-B21/C21</f>
+        <f t="shared" si="0"/>
         <v>0.53846153846153844</v>
       </c>
       <c r="E21" s="11" t="s">
@@ -2890,7 +2890,7 @@
         <v>63</v>
       </c>
       <c r="D22" s="12">
-        <f>1-B22/C22</f>
+        <f t="shared" si="0"/>
         <v>0.77777777777777779</v>
       </c>
       <c r="E22" s="11" t="s">
@@ -2908,7 +2908,7 @@
         <v>39</v>
       </c>
       <c r="D23" s="12">
-        <f>1-B23/C23</f>
+        <f t="shared" si="0"/>
         <v>0.84615384615384615</v>
       </c>
       <c r="E23" s="11" t="s">
@@ -2926,7 +2926,7 @@
         <v>362</v>
       </c>
       <c r="D24" s="12">
-        <f>1-B24/C24</f>
+        <f t="shared" si="0"/>
         <v>0.70994475138121549</v>
       </c>
       <c r="E24" s="11" t="s">
@@ -2944,7 +2944,7 @@
         <v>289</v>
       </c>
       <c r="D25" s="12">
-        <f>1-B25/C25</f>
+        <f t="shared" si="0"/>
         <v>0.48788927335640142</v>
       </c>
       <c r="E25" s="11" t="s">
@@ -2962,7 +2962,7 @@
         <v>58</v>
       </c>
       <c r="D26" s="12">
-        <f>1-B26/C26</f>
+        <f t="shared" si="0"/>
         <v>0.82758620689655171</v>
       </c>
       <c r="E26" s="11" t="s">
@@ -2980,7 +2980,7 @@
         <v>79</v>
       </c>
       <c r="D27" s="12">
-        <f>1-B27/C27</f>
+        <f t="shared" si="0"/>
         <v>0.36708860759493667</v>
       </c>
       <c r="E27" s="11" t="s">
@@ -2998,7 +2998,7 @@
         <v>182</v>
       </c>
       <c r="D28" s="12">
-        <f>1-B28/C28</f>
+        <f t="shared" si="0"/>
         <v>0.68131868131868134</v>
       </c>
       <c r="E28" s="11" t="s">
@@ -3016,7 +3016,7 @@
         <v>307</v>
       </c>
       <c r="D29" s="12">
-        <f>1-B29/C29</f>
+        <f t="shared" si="0"/>
         <v>0.83387622149837137</v>
       </c>
       <c r="E29" s="11" t="s">
@@ -3034,7 +3034,7 @@
         <v>48</v>
       </c>
       <c r="D30" s="12">
-        <f>1-B30/C30</f>
+        <f t="shared" si="0"/>
         <v>0.79166666666666663</v>
       </c>
       <c r="E30" s="11" t="s">
@@ -3052,7 +3052,7 @@
         <v>33</v>
       </c>
       <c r="D31" s="12">
-        <f>1-B31/C31</f>
+        <f t="shared" si="0"/>
         <v>0.90909090909090906</v>
       </c>
       <c r="E31" s="11" t="s">
@@ -3070,7 +3070,7 @@
         <v>185</v>
       </c>
       <c r="D32" s="12">
-        <f>1-B32/C32</f>
+        <f t="shared" si="0"/>
         <v>0.61621621621621614</v>
       </c>
       <c r="E32" s="11" t="s">
@@ -3088,7 +3088,7 @@
         <v>245</v>
       </c>
       <c r="D33" s="12">
-        <f>1-B33/C33</f>
+        <f t="shared" si="0"/>
         <v>0.88163265306122451</v>
       </c>
       <c r="E33" s="11" t="s">
@@ -3106,7 +3106,7 @@
         <v>79</v>
       </c>
       <c r="D34" s="12">
-        <f>1-B34/C34</f>
+        <f t="shared" si="0"/>
         <v>0.77215189873417722</v>
       </c>
       <c r="E34" s="11" t="s">
@@ -3124,7 +3124,7 @@
         <v>41</v>
       </c>
       <c r="D35" s="12">
-        <f>1-B35/C35</f>
+        <f t="shared" si="0"/>
         <v>0.85365853658536583</v>
       </c>
       <c r="E35" s="11" t="s">

</xml_diff>